<commit_message>
Updating table names and dataset name as requested by Fabian0 9-24-2026
</commit_message>
<xml_diff>
--- a/htan2-data-release-pipeline/medallion_architecture/gold2isbcgc/log/Metadata_Table_Descriptions_R8.xlsx
+++ b/htan2-data-release-pipeline/medallion_architecture/gold2isbcgc/log/Metadata_Table_Descriptions_R8.xlsx
@@ -513,22 +513,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>htan2-dcc.htan2_isbcgcbq_current_release.HTAN2_MultiplexMicroscopyLevel2_File_Metadata</t>
+          <t>htan2-dcc.htan2_isbcgcbq_current_release.MultiplexMicroscopyLevel2_File_Metadata</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>HTAN2 and HTAN2_versioned</t>
+          <t>HTAN2</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>HTAN2_MultiplexMicroscopyLevel2_File_Metadata_current</t>
+          <t>MultiplexMicroscopyLevel2_File_Metadata_current</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>HTAN2_MultiplexMicroscopyLevel2_File_Metadata_r8</t>
+          <t>MultiplexMicroscopyLevel2_File_Metadata_r8</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -591,22 +591,22 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>htan2-dcc.htan2_isbcgcbq_current_release.HTAN2_SpatialLevel3_File_Metadata</t>
+          <t>htan2-dcc.htan2_isbcgcbq_current_release.SpatialLevel3_File_Metadata</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>HTAN2 and HTAN2_versioned</t>
+          <t>HTAN2</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>HTAN2_SpatialLevel3_File_Metadata_current</t>
+          <t>SpatialLevel3_File_Metadata_current</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>HTAN2_SpatialLevel3_File_Metadata_r8</t>
+          <t>SpatialLevel3_File_Metadata_r8</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -669,22 +669,22 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>htan2-dcc.htan2_isbcgcbq_current_release.HTAN2_scRNALevel1_File_Metadata</t>
+          <t>htan2-dcc.htan2_isbcgcbq_current_release.scRNALevel1_File_Metadata</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>HTAN2 and HTAN2_versioned</t>
+          <t>HTAN2</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>HTAN2_scRNALevel1_File_Metadata_current</t>
+          <t>scRNALevel1_File_Metadata_current</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>HTAN2_scRNALevel1_File_Metadata_r8</t>
+          <t>scRNALevel1_File_Metadata_r8</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -747,22 +747,22 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>htan2-dcc.htan2_isbcgcbq_current_release.HTAN2_scRNALevel2_File_Metadata</t>
+          <t>htan2-dcc.htan2_isbcgcbq_current_release.scRNALevel2_File_Metadata</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>HTAN2 and HTAN2_versioned</t>
+          <t>HTAN2</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>HTAN2_scRNALevel2_File_Metadata_current</t>
+          <t>scRNALevel2_File_Metadata_current</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>HTAN2_scRNALevel2_File_Metadata_r8</t>
+          <t>scRNALevel2_File_Metadata_r8</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -825,22 +825,22 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>htan2-dcc.htan2_isbcgcbq_current_release.HTAN2_Biospecimen_Sample_Metadata</t>
+          <t>htan2-dcc.htan2_isbcgcbq_current_release.Biospecimen_Sample_Metadata</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>HTAN2 and HTAN2_versioned</t>
+          <t>HTAN2</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>HTAN2_Biospecimen_Sample_Metadata_current</t>
+          <t>Biospecimen_Sample_Metadata_current</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>HTAN2_Biospecimen_Sample_Metadata_r8</t>
+          <t>Biospecimen_Sample_Metadata_r8</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -903,22 +903,22 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>htan2-dcc.htan2_isbcgcbq_current_release.HTAN2_ChannelMetadata_File_Metadata</t>
+          <t>htan2-dcc.htan2_isbcgcbq_current_release.ChannelMetadata_File_Metadata</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>HTAN2 and HTAN2_versioned</t>
+          <t>HTAN2</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>HTAN2_ChannelMetadata_File_Metadata_current</t>
+          <t>ChannelMetadata_File_Metadata_current</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>HTAN2_ChannelMetadata_File_Metadata_r8</t>
+          <t>ChannelMetadata_File_Metadata_r8</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -981,22 +981,22 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>htan2-dcc.htan2_isbcgcbq_current_release.HTAN2_Demographics_Clinical_Metadata</t>
+          <t>htan2-dcc.htan2_isbcgcbq_current_release.Demographics_Clinical_Metadata</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>HTAN2 and HTAN2_versioned</t>
+          <t>HTAN2</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>HTAN2_Demographics_Clinical_Metadata_current</t>
+          <t>Demographics_Clinical_Metadata_current</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>HTAN2_Demographics_Clinical_Metadata_r8</t>
+          <t>Demographics_Clinical_Metadata_r8</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1059,22 +1059,22 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>htan2-dcc.htan2_isbcgcbq_current_release.HTAN2_Diagnosis_Clinical_Metadata</t>
+          <t>htan2-dcc.htan2_isbcgcbq_current_release.Diagnosis_Clinical_Metadata</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>HTAN2 and HTAN2_versioned</t>
+          <t>HTAN2</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>HTAN2_Diagnosis_Clinical_Metadata_current</t>
+          <t>Diagnosis_Clinical_Metadata_current</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>HTAN2_Diagnosis_Clinical_Metadata_r8</t>
+          <t>Diagnosis_Clinical_Metadata_r8</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1137,22 +1137,22 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>htan2-dcc.htan2_isbcgcbq_current_release.HTAN2_Exposure_Clinical_Metadata</t>
+          <t>htan2-dcc.htan2_isbcgcbq_current_release.Exposure_Clinical_Metadata</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>HTAN2 and HTAN2_versioned</t>
+          <t>HTAN2</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>HTAN2_Exposure_Clinical_Metadata_current</t>
+          <t>Exposure_Clinical_Metadata_current</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>HTAN2_Exposure_Clinical_Metadata_r8</t>
+          <t>Exposure_Clinical_Metadata_r8</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1215,22 +1215,22 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>htan2-dcc.htan2_isbcgcbq_current_release.HTAN2_FamilyHistory_Clinical_Metadata</t>
+          <t>htan2-dcc.htan2_isbcgcbq_current_release.FamilyHistory_Clinical_Metadata</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>HTAN2 and HTAN2_versioned</t>
+          <t>HTAN2</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>HTAN2_FamilyHistory_Clinical_Metadata_current</t>
+          <t>FamilyHistory_Clinical_Metadata_current</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>HTAN2_FamilyHistory_Clinical_Metadata_r8</t>
+          <t>FamilyHistory_Clinical_Metadata_r8</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1293,22 +1293,22 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>htan2-dcc.htan2_isbcgcbq_current_release.HTAN2_FollowUp_Clinical_Metadata</t>
+          <t>htan2-dcc.htan2_isbcgcbq_current_release.FollowUp_Clinical_Metadata</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>HTAN2 and HTAN2_versioned</t>
+          <t>HTAN2</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>HTAN2_FollowUp_Clinical_Metadata_current</t>
+          <t>FollowUp_Clinical_Metadata_current</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>HTAN2_FollowUp_Clinical_Metadata_r8</t>
+          <t>FollowUp_Clinical_Metadata_r8</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1371,22 +1371,22 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>htan2-dcc.htan2_isbcgcbq_current_release.HTAN2_MolecularTest_Clinical_Metadata</t>
+          <t>htan2-dcc.htan2_isbcgcbq_current_release.MolecularTest_Clinical_Metadata</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>HTAN2 and HTAN2_versioned</t>
+          <t>HTAN2</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>HTAN2_MolecularTest_Clinical_Metadata_current</t>
+          <t>MolecularTest_Clinical_Metadata_current</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>HTAN2_MolecularTest_Clinical_Metadata_r8</t>
+          <t>MolecularTest_Clinical_Metadata_r8</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1449,22 +1449,22 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>htan2-dcc.htan2_isbcgcbq_current_release.HTAN2_SpatialPanel_File_Metadata</t>
+          <t>htan2-dcc.htan2_isbcgcbq_current_release.SpatialPanel_File_Metadata</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>HTAN2 and HTAN2_versioned</t>
+          <t>HTAN2</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>HTAN2_SpatialPanel_File_Metadata_current</t>
+          <t>SpatialPanel_File_Metadata_current</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>HTAN2_SpatialPanel_File_Metadata_r8</t>
+          <t>SpatialPanel_File_Metadata_r8</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1527,22 +1527,22 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>htan2-dcc.htan2_isbcgcbq_current_release.HTAN2_Therapy_Clinical_Metadata</t>
+          <t>htan2-dcc.htan2_isbcgcbq_current_release.Therapy_Clinical_Metadata</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>HTAN2 and HTAN2_versioned</t>
+          <t>HTAN2</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>HTAN2_Therapy_Clinical_Metadata_current</t>
+          <t>Therapy_Clinical_Metadata_current</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>HTAN2_Therapy_Clinical_Metadata_r8</t>
+          <t>Therapy_Clinical_Metadata_r8</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1605,22 +1605,22 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>htan2-dcc.htan2_isbcgcbq_current_release.HTAN2_VitalStatus_Clinical_Metadata</t>
+          <t>htan2-dcc.htan2_isbcgcbq_current_release.VitalStatus_Clinical_Metadata</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>HTAN2 and HTAN2_versioned</t>
+          <t>HTAN2</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>HTAN2_VitalStatus_Clinical_Metadata_current</t>
+          <t>VitalStatus_Clinical_Metadata_current</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>HTAN2_VitalStatus_Clinical_Metadata_r8</t>
+          <t>VitalStatus_Clinical_Metadata_r8</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1683,22 +1683,22 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>htan2-dcc.htan2_isbcgcbq_current_release.HTAN2_Data_Model_Schema</t>
+          <t>htan2-dcc.htan2_isbcgcbq_current_release.Data_Model_v1_5_0_Schema</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>HTAN2 and HTAN2_versioned</t>
+          <t>HTAN2</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>HTAN2_Data_Model_Schema_current</t>
+          <t>Data_Model_v1_5_0_Schema_current</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>HTAN2_Data_Model_Schema_r8</t>
+          <t>Data_Model_v1_5_0_Schema_r8</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1761,22 +1761,22 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>htan2-dcc.htan2_isbcgcbq_current_release.HTAN2_ID_Provenance_Chain</t>
+          <t>htan2-dcc.htan2_isbcgcbq_current_release.ID_Provenance_Chain</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>HTAN2 and HTAN2_versioned</t>
+          <t>HTAN2</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>HTAN2_ID_Provenance_Chain_current</t>
+          <t>ID_Provenance_Chain_current</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>HTAN2_ID_Provenance_Chain_r8</t>
+          <t>ID_Provenance_Chain_r8</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">

</xml_diff>

<commit_message>
Update Tables for Isb-cgc
Add new Data_Release and CRDC_Release Columns.
- Data release column is based on Status_Folder_Name 
- Drop Status_Folder_Name
-Add missing descriptions for new columns
-Add cleanup suggested by Fabian (remove quotes, brackets from HTAN_Parent_ID)
</commit_message>
<xml_diff>
--- a/htan2-data-release-pipeline/medallion_architecture/gold2isbcgc/log/Metadata_Table_Descriptions_R8.xlsx
+++ b/htan2-data-release-pipeline/medallion_architecture/gold2isbcgc/log/Metadata_Table_Descriptions_R8.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P18"/>
+  <dimension ref="A1:P17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1293,7 +1293,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>htan2-dcc.htan2_isbcgcbq_current_release.FollowUp_Clinical_Metadata</t>
+          <t>htan2-dcc.htan2_isbcgcbq_current_release.MolecularTest_Clinical_Metadata</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1303,22 +1303,22 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>FollowUp_Clinical_Metadata_current</t>
+          <t>MolecularTest_Clinical_Metadata_current</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>FollowUp_Clinical_Metadata_r8</t>
+          <t>MolecularTest_Clinical_Metadata_r8</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>This table contains the clinical metadata for Follow Up data extracted from HTAN Phase 2 Synapse projects in July 2026 and corresponds to HTAN2 Data Release 8.0.</t>
+          <t>This table contains the clinical metadata for Molecular Test data extracted from HTAN Phase 2 Synapse projects in July 2026 and corresponds to HTAN2 Data Release 8.0.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>HTAN PHASE 2 CLINICAL METADATA FOR FOLLOW UP</t>
+          <t>HTAN PHASE 2 CLINICAL METADATA FOR MOLECULAR TEST</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1362,16 +1362,16 @@
         </is>
       </c>
       <c r="O12" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="P12" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>htan2-dcc.htan2_isbcgcbq_current_release.MolecularTest_Clinical_Metadata</t>
+          <t>htan2-dcc.htan2_isbcgcbq_current_release.SpatialPanel_File_Metadata</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1381,22 +1381,22 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MolecularTest_Clinical_Metadata_current</t>
+          <t>SpatialPanel_File_Metadata_current</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>MolecularTest_Clinical_Metadata_r8</t>
+          <t>SpatialPanel_File_Metadata_r8</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>This table contains the clinical metadata for Molecular Test data extracted from HTAN Phase 2 Synapse projects in July 2026 and corresponds to HTAN2 Data Release 8.0.</t>
+          <t>This table contains the file metadata for Spatial Panel data extracted from HTAN Phase 2 Synapse projects in July 2026 and corresponds to HTAN2 Data Release 8.0.</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>HTAN PHASE 2 CLINICAL METADATA FOR MOLECULAR TEST</t>
+          <t>HTAN PHASE 2 FILE METADATA FOR SPATIAL PANEL</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1416,7 +1416,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>clinical_biospecimen_data</t>
+          <t>metadata</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>clinical_data</t>
+          <t>file_metadata</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1440,16 +1440,16 @@
         </is>
       </c>
       <c r="O13" t="n">
-        <v>10</v>
+        <v>6532</v>
       </c>
       <c r="P13" t="n">
-        <v>10</v>
+        <v>6532</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>htan2-dcc.htan2_isbcgcbq_current_release.SpatialPanel_File_Metadata</t>
+          <t>htan2-dcc.htan2_isbcgcbq_current_release.Therapy_Clinical_Metadata</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1459,22 +1459,22 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>SpatialPanel_File_Metadata_current</t>
+          <t>Therapy_Clinical_Metadata_current</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>SpatialPanel_File_Metadata_r8</t>
+          <t>Therapy_Clinical_Metadata_r8</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>This table contains the file metadata for Spatial Panel data extracted from HTAN Phase 2 Synapse projects in July 2026 and corresponds to HTAN2 Data Release 8.0.</t>
+          <t>This table contains the clinical metadata for Therapy data extracted from HTAN Phase 2 Synapse projects in July 2026 and corresponds to HTAN2 Data Release 8.0.</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>HTAN PHASE 2 FILE METADATA FOR SPATIAL PANEL</t>
+          <t>HTAN PHASE 2 CLINICAL METADATA FOR THERAPY</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1494,7 +1494,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>metadata</t>
+          <t>clinical_biospecimen_data</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1509,7 +1509,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>file_metadata</t>
+          <t>clinical_data</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1518,16 +1518,16 @@
         </is>
       </c>
       <c r="O14" t="n">
-        <v>6532</v>
+        <v>11</v>
       </c>
       <c r="P14" t="n">
-        <v>6532</v>
+        <v>11</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>htan2-dcc.htan2_isbcgcbq_current_release.Therapy_Clinical_Metadata</t>
+          <t>htan2-dcc.htan2_isbcgcbq_current_release.VitalStatus_Clinical_Metadata</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1537,22 +1537,22 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Therapy_Clinical_Metadata_current</t>
+          <t>VitalStatus_Clinical_Metadata_current</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Therapy_Clinical_Metadata_r8</t>
+          <t>VitalStatus_Clinical_Metadata_r8</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>This table contains the clinical metadata for Therapy data extracted from HTAN Phase 2 Synapse projects in July 2026 and corresponds to HTAN2 Data Release 8.0.</t>
+          <t>This table contains the clinical metadata for Vital Status data extracted from HTAN Phase 2 Synapse projects in July 2026 and corresponds to HTAN2 Data Release 8.0.</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>HTAN PHASE 2 CLINICAL METADATA FOR THERAPY</t>
+          <t>HTAN PHASE 2 CLINICAL METADATA FOR VITAL STATUS</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1605,7 +1605,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>htan2-dcc.htan2_isbcgcbq_current_release.VitalStatus_Clinical_Metadata</t>
+          <t>htan2-dcc.htan2_isbcgcbq_current_release.Data_Model_v1_5_0_Schema</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1615,22 +1615,22 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>VitalStatus_Clinical_Metadata_current</t>
+          <t>Data_Model_v1_5_0_Schema_current</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>VitalStatus_Clinical_Metadata_r8</t>
+          <t>Data_Model_v1_5_0_Schema_r8</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>This table contains the clinical metadata for Vital Status data extracted from HTAN Phase 2 Synapse projects in July 2026 and corresponds to HTAN2 Data Release 8.0.</t>
+          <t>Data was extracted from the the HTAN Phase 2 Data Model v1.5.0 in July 2026. For more details see: https://htan2-data-model.readthedocs.io/en/main/</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>HTAN PHASE 2 CLINICAL METADATA FOR VITAL STATUS</t>
+          <t>HTAN PHASE 2 DATA MODEL SCHEMA (v1.5.0)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1650,7 +1650,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>clinical_biospecimen_data</t>
+          <t>metadata</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>clinical_data</t>
+          <t>data_dictionary</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1674,16 +1674,16 @@
         </is>
       </c>
       <c r="O16" t="n">
-        <v>11</v>
+        <v>527</v>
       </c>
       <c r="P16" t="n">
-        <v>11</v>
+        <v>527</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>htan2-dcc.htan2_isbcgcbq_current_release.Data_Model_v1_5_0_Schema</t>
+          <t>htan2-dcc.htan2_isbcgcbq_current_release.ID_Provenance_Chain</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1693,22 +1693,22 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Data_Model_v1_5_0_Schema_current</t>
+          <t>ID_Provenance_Chain_current</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Data_Model_v1_5_0_Schema_r8</t>
+          <t>ID_Provenance_Chain_r8</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Data was extracted from the the HTAN Phase 2 Data Model v1.5.0 in July 2026. For more details see: https://htan2-data-model.readthedocs.io/en/main/</t>
+          <t>This table contains biospecimen and participant IDs for each HTAN2 data file. This table was created in July 2026 and uploaded July 2026 and corresponds to the HTAN Phase 2 Data Release 8.0.</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>HTAN PHASE 2 DATA MODEL SCHEMA (v1.5.0)</t>
+          <t>HTAN PHASE 2 ID PROVENANCE CHAIN</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1743,7 +1743,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>data_dictionary</t>
+          <t>file_metadata</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1752,87 +1752,9 @@
         </is>
       </c>
       <c r="O17" t="n">
-        <v>527</v>
+        <v>65</v>
       </c>
       <c r="P17" t="n">
-        <v>527</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>htan2-dcc.htan2_isbcgcbq_current_release.ID_Provenance_Chain</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>HTAN2</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>ID_Provenance_Chain_current</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>ID_Provenance_Chain_r8</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>This table contains biospecimen and participant IDs for each HTAN2 data file. This table was created in July 2026 and uploaded July 2026 and corresponds to the HTAN Phase 2 Data Release 8.0.</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>HTAN PHASE 2 ID PROVENANCE CHAIN</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>current</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>htan2</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>metadata</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>NULL</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>htan</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>file_metadata</t>
-        </is>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>r8</t>
-        </is>
-      </c>
-      <c r="O18" t="n">
-        <v>65</v>
-      </c>
-      <c r="P18" t="n">
         <v>65</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Revert "Update Tables for Isb-cgc"
This reverts commit ed3bc0f9689940251f4626f9485a57f212cde8aa.
</commit_message>
<xml_diff>
--- a/htan2-data-release-pipeline/medallion_architecture/gold2isbcgc/log/Metadata_Table_Descriptions_R8.xlsx
+++ b/htan2-data-release-pipeline/medallion_architecture/gold2isbcgc/log/Metadata_Table_Descriptions_R8.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P17"/>
+  <dimension ref="A1:P18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1293,7 +1293,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>htan2-dcc.htan2_isbcgcbq_current_release.MolecularTest_Clinical_Metadata</t>
+          <t>htan2-dcc.htan2_isbcgcbq_current_release.FollowUp_Clinical_Metadata</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1303,22 +1303,22 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MolecularTest_Clinical_Metadata_current</t>
+          <t>FollowUp_Clinical_Metadata_current</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>MolecularTest_Clinical_Metadata_r8</t>
+          <t>FollowUp_Clinical_Metadata_r8</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>This table contains the clinical metadata for Molecular Test data extracted from HTAN Phase 2 Synapse projects in July 2026 and corresponds to HTAN2 Data Release 8.0.</t>
+          <t>This table contains the clinical metadata for Follow Up data extracted from HTAN Phase 2 Synapse projects in July 2026 and corresponds to HTAN2 Data Release 8.0.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>HTAN PHASE 2 CLINICAL METADATA FOR MOLECULAR TEST</t>
+          <t>HTAN PHASE 2 CLINICAL METADATA FOR FOLLOW UP</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1362,16 +1362,16 @@
         </is>
       </c>
       <c r="O12" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="P12" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>htan2-dcc.htan2_isbcgcbq_current_release.SpatialPanel_File_Metadata</t>
+          <t>htan2-dcc.htan2_isbcgcbq_current_release.MolecularTest_Clinical_Metadata</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1381,22 +1381,22 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>SpatialPanel_File_Metadata_current</t>
+          <t>MolecularTest_Clinical_Metadata_current</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>SpatialPanel_File_Metadata_r8</t>
+          <t>MolecularTest_Clinical_Metadata_r8</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>This table contains the file metadata for Spatial Panel data extracted from HTAN Phase 2 Synapse projects in July 2026 and corresponds to HTAN2 Data Release 8.0.</t>
+          <t>This table contains the clinical metadata for Molecular Test data extracted from HTAN Phase 2 Synapse projects in July 2026 and corresponds to HTAN2 Data Release 8.0.</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>HTAN PHASE 2 FILE METADATA FOR SPATIAL PANEL</t>
+          <t>HTAN PHASE 2 CLINICAL METADATA FOR MOLECULAR TEST</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1416,7 +1416,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>metadata</t>
+          <t>clinical_biospecimen_data</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>file_metadata</t>
+          <t>clinical_data</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1440,16 +1440,16 @@
         </is>
       </c>
       <c r="O13" t="n">
-        <v>6532</v>
+        <v>10</v>
       </c>
       <c r="P13" t="n">
-        <v>6532</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>htan2-dcc.htan2_isbcgcbq_current_release.Therapy_Clinical_Metadata</t>
+          <t>htan2-dcc.htan2_isbcgcbq_current_release.SpatialPanel_File_Metadata</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1459,22 +1459,22 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Therapy_Clinical_Metadata_current</t>
+          <t>SpatialPanel_File_Metadata_current</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Therapy_Clinical_Metadata_r8</t>
+          <t>SpatialPanel_File_Metadata_r8</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>This table contains the clinical metadata for Therapy data extracted from HTAN Phase 2 Synapse projects in July 2026 and corresponds to HTAN2 Data Release 8.0.</t>
+          <t>This table contains the file metadata for Spatial Panel data extracted from HTAN Phase 2 Synapse projects in July 2026 and corresponds to HTAN2 Data Release 8.0.</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>HTAN PHASE 2 CLINICAL METADATA FOR THERAPY</t>
+          <t>HTAN PHASE 2 FILE METADATA FOR SPATIAL PANEL</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1494,7 +1494,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>clinical_biospecimen_data</t>
+          <t>metadata</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1509,7 +1509,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>clinical_data</t>
+          <t>file_metadata</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1518,16 +1518,16 @@
         </is>
       </c>
       <c r="O14" t="n">
-        <v>11</v>
+        <v>6532</v>
       </c>
       <c r="P14" t="n">
-        <v>11</v>
+        <v>6532</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>htan2-dcc.htan2_isbcgcbq_current_release.VitalStatus_Clinical_Metadata</t>
+          <t>htan2-dcc.htan2_isbcgcbq_current_release.Therapy_Clinical_Metadata</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1537,22 +1537,22 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>VitalStatus_Clinical_Metadata_current</t>
+          <t>Therapy_Clinical_Metadata_current</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>VitalStatus_Clinical_Metadata_r8</t>
+          <t>Therapy_Clinical_Metadata_r8</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>This table contains the clinical metadata for Vital Status data extracted from HTAN Phase 2 Synapse projects in July 2026 and corresponds to HTAN2 Data Release 8.0.</t>
+          <t>This table contains the clinical metadata for Therapy data extracted from HTAN Phase 2 Synapse projects in July 2026 and corresponds to HTAN2 Data Release 8.0.</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>HTAN PHASE 2 CLINICAL METADATA FOR VITAL STATUS</t>
+          <t>HTAN PHASE 2 CLINICAL METADATA FOR THERAPY</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1605,7 +1605,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>htan2-dcc.htan2_isbcgcbq_current_release.Data_Model_v1_5_0_Schema</t>
+          <t>htan2-dcc.htan2_isbcgcbq_current_release.VitalStatus_Clinical_Metadata</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1615,22 +1615,22 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Data_Model_v1_5_0_Schema_current</t>
+          <t>VitalStatus_Clinical_Metadata_current</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Data_Model_v1_5_0_Schema_r8</t>
+          <t>VitalStatus_Clinical_Metadata_r8</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Data was extracted from the the HTAN Phase 2 Data Model v1.5.0 in July 2026. For more details see: https://htan2-data-model.readthedocs.io/en/main/</t>
+          <t>This table contains the clinical metadata for Vital Status data extracted from HTAN Phase 2 Synapse projects in July 2026 and corresponds to HTAN2 Data Release 8.0.</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>HTAN PHASE 2 DATA MODEL SCHEMA (v1.5.0)</t>
+          <t>HTAN PHASE 2 CLINICAL METADATA FOR VITAL STATUS</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1650,7 +1650,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>metadata</t>
+          <t>clinical_biospecimen_data</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>data_dictionary</t>
+          <t>clinical_data</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1674,87 +1674,165 @@
         </is>
       </c>
       <c r="O16" t="n">
-        <v>527</v>
+        <v>11</v>
       </c>
       <c r="P16" t="n">
-        <v>527</v>
+        <v>11</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>htan2-dcc.htan2_isbcgcbq_current_release.Data_Model_v1_5_0_Schema</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>HTAN2</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Data_Model_v1_5_0_Schema_current</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Data_Model_v1_5_0_Schema_r8</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Data was extracted from the the HTAN Phase 2 Data Model v1.5.0 in July 2026. For more details see: https://htan2-data-model.readthedocs.io/en/main/</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>HTAN PHASE 2 DATA MODEL SCHEMA (v1.5.0)</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>htan2</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>metadata</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>htan</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>data_dictionary</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>r8</t>
+        </is>
+      </c>
+      <c r="O17" t="n">
+        <v>527</v>
+      </c>
+      <c r="P17" t="n">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>htan2-dcc.htan2_isbcgcbq_current_release.ID_Provenance_Chain</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>HTAN2</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>ID_Provenance_Chain_current</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>ID_Provenance_Chain_r8</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>This table contains biospecimen and participant IDs for each HTAN2 data file. This table was created in July 2026 and uploaded July 2026 and corresponds to the HTAN Phase 2 Data Release 8.0.</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>HTAN PHASE 2 ID PROVENANCE CHAIN</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>current</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>htan2</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>metadata</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t>NULL</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>htan</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
+      <c r="M18" t="inlineStr">
         <is>
           <t>file_metadata</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr">
+      <c r="N18" t="inlineStr">
         <is>
           <t>r8</t>
         </is>
       </c>
-      <c r="O17" t="n">
+      <c r="O18" t="n">
         <v>65</v>
       </c>
-      <c r="P17" t="n">
+      <c r="P18" t="n">
         <v>65</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update isb-cgc staged tables in htan2-dcc
Update Tables for isb-cgc
Add new Data_Release and CRDC_Release Columns.
- Data release column is based on Status_Folder_Name 
- Drop Status_Folder_Name
-Add missing descriptions for new columns
-Add cleanup suggested by Fabian (remove quotes, brackets from HTAN_Parent_ID)
</commit_message>
<xml_diff>
--- a/htan2-data-release-pipeline/medallion_architecture/gold2isbcgc/log/Metadata_Table_Descriptions_R8.xlsx
+++ b/htan2-data-release-pipeline/medallion_architecture/gold2isbcgc/log/Metadata_Table_Descriptions_R8.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P18"/>
+  <dimension ref="A1:P17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1293,7 +1293,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>htan2-dcc.htan2_isbcgcbq_current_release.FollowUp_Clinical_Metadata</t>
+          <t>htan2-dcc.htan2_isbcgcbq_current_release.MolecularTest_Clinical_Metadata</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1303,22 +1303,22 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>FollowUp_Clinical_Metadata_current</t>
+          <t>MolecularTest_Clinical_Metadata_current</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>FollowUp_Clinical_Metadata_r8</t>
+          <t>MolecularTest_Clinical_Metadata_r8</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>This table contains the clinical metadata for Follow Up data extracted from HTAN Phase 2 Synapse projects in July 2026 and corresponds to HTAN2 Data Release 8.0.</t>
+          <t>This table contains the clinical metadata for Molecular Test data extracted from HTAN Phase 2 Synapse projects in July 2026 and corresponds to HTAN2 Data Release 8.0.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>HTAN PHASE 2 CLINICAL METADATA FOR FOLLOW UP</t>
+          <t>HTAN PHASE 2 CLINICAL METADATA FOR MOLECULAR TEST</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1362,16 +1362,16 @@
         </is>
       </c>
       <c r="O12" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="P12" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>htan2-dcc.htan2_isbcgcbq_current_release.MolecularTest_Clinical_Metadata</t>
+          <t>htan2-dcc.htan2_isbcgcbq_current_release.SpatialPanel_File_Metadata</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1381,22 +1381,22 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MolecularTest_Clinical_Metadata_current</t>
+          <t>SpatialPanel_File_Metadata_current</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>MolecularTest_Clinical_Metadata_r8</t>
+          <t>SpatialPanel_File_Metadata_r8</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>This table contains the clinical metadata for Molecular Test data extracted from HTAN Phase 2 Synapse projects in July 2026 and corresponds to HTAN2 Data Release 8.0.</t>
+          <t>This table contains the file metadata for Spatial Panel data extracted from HTAN Phase 2 Synapse projects in July 2026 and corresponds to HTAN2 Data Release 8.0.</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>HTAN PHASE 2 CLINICAL METADATA FOR MOLECULAR TEST</t>
+          <t>HTAN PHASE 2 FILE METADATA FOR SPATIAL PANEL</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1416,7 +1416,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>clinical_biospecimen_data</t>
+          <t>metadata</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>clinical_data</t>
+          <t>file_metadata</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1440,16 +1440,16 @@
         </is>
       </c>
       <c r="O13" t="n">
-        <v>10</v>
+        <v>6532</v>
       </c>
       <c r="P13" t="n">
-        <v>10</v>
+        <v>6532</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>htan2-dcc.htan2_isbcgcbq_current_release.SpatialPanel_File_Metadata</t>
+          <t>htan2-dcc.htan2_isbcgcbq_current_release.Therapy_Clinical_Metadata</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1459,22 +1459,22 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>SpatialPanel_File_Metadata_current</t>
+          <t>Therapy_Clinical_Metadata_current</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>SpatialPanel_File_Metadata_r8</t>
+          <t>Therapy_Clinical_Metadata_r8</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>This table contains the file metadata for Spatial Panel data extracted from HTAN Phase 2 Synapse projects in July 2026 and corresponds to HTAN2 Data Release 8.0.</t>
+          <t>This table contains the clinical metadata for Therapy data extracted from HTAN Phase 2 Synapse projects in July 2026 and corresponds to HTAN2 Data Release 8.0.</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>HTAN PHASE 2 FILE METADATA FOR SPATIAL PANEL</t>
+          <t>HTAN PHASE 2 CLINICAL METADATA FOR THERAPY</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1494,7 +1494,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>metadata</t>
+          <t>clinical_biospecimen_data</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1509,7 +1509,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>file_metadata</t>
+          <t>clinical_data</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1518,16 +1518,16 @@
         </is>
       </c>
       <c r="O14" t="n">
-        <v>6532</v>
+        <v>11</v>
       </c>
       <c r="P14" t="n">
-        <v>6532</v>
+        <v>11</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>htan2-dcc.htan2_isbcgcbq_current_release.Therapy_Clinical_Metadata</t>
+          <t>htan2-dcc.htan2_isbcgcbq_current_release.VitalStatus_Clinical_Metadata</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1537,22 +1537,22 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Therapy_Clinical_Metadata_current</t>
+          <t>VitalStatus_Clinical_Metadata_current</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Therapy_Clinical_Metadata_r8</t>
+          <t>VitalStatus_Clinical_Metadata_r8</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>This table contains the clinical metadata for Therapy data extracted from HTAN Phase 2 Synapse projects in July 2026 and corresponds to HTAN2 Data Release 8.0.</t>
+          <t>This table contains the clinical metadata for Vital Status data extracted from HTAN Phase 2 Synapse projects in July 2026 and corresponds to HTAN2 Data Release 8.0.</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>HTAN PHASE 2 CLINICAL METADATA FOR THERAPY</t>
+          <t>HTAN PHASE 2 CLINICAL METADATA FOR VITAL STATUS</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1605,7 +1605,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>htan2-dcc.htan2_isbcgcbq_current_release.VitalStatus_Clinical_Metadata</t>
+          <t>htan2-dcc.htan2_isbcgcbq_current_release.Data_Model_v1_5_0_Schema</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1615,22 +1615,22 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>VitalStatus_Clinical_Metadata_current</t>
+          <t>Data_Model_v1_5_0_Schema_current</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>VitalStatus_Clinical_Metadata_r8</t>
+          <t>Data_Model_v1_5_0_Schema_r8</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>This table contains the clinical metadata for Vital Status data extracted from HTAN Phase 2 Synapse projects in July 2026 and corresponds to HTAN2 Data Release 8.0.</t>
+          <t>Data was extracted from the the HTAN Phase 2 Data Model v1.5.0 in July 2026. For more details see: https://htan2-data-model.readthedocs.io/en/main/</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>HTAN PHASE 2 CLINICAL METADATA FOR VITAL STATUS</t>
+          <t>HTAN PHASE 2 DATA MODEL SCHEMA (v1.5.0)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1650,7 +1650,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>clinical_biospecimen_data</t>
+          <t>metadata</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>clinical_data</t>
+          <t>data_dictionary</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1674,16 +1674,16 @@
         </is>
       </c>
       <c r="O16" t="n">
-        <v>11</v>
+        <v>527</v>
       </c>
       <c r="P16" t="n">
-        <v>11</v>
+        <v>527</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>htan2-dcc.htan2_isbcgcbq_current_release.Data_Model_v1_5_0_Schema</t>
+          <t>htan2-dcc.htan2_isbcgcbq_current_release.ID_Provenance_Chain</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1693,22 +1693,22 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Data_Model_v1_5_0_Schema_current</t>
+          <t>ID_Provenance_Chain_current</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Data_Model_v1_5_0_Schema_r8</t>
+          <t>ID_Provenance_Chain_r8</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Data was extracted from the the HTAN Phase 2 Data Model v1.5.0 in July 2026. For more details see: https://htan2-data-model.readthedocs.io/en/main/</t>
+          <t>This table contains biospecimen and participant IDs for each HTAN2 data file. This table was created in July 2026 and uploaded July 2026 and corresponds to the HTAN Phase 2 Data Release 8.0.</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>HTAN PHASE 2 DATA MODEL SCHEMA (v1.5.0)</t>
+          <t>HTAN PHASE 2 ID PROVENANCE CHAIN</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1743,7 +1743,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>data_dictionary</t>
+          <t>file_metadata</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1752,87 +1752,9 @@
         </is>
       </c>
       <c r="O17" t="n">
-        <v>527</v>
+        <v>65</v>
       </c>
       <c r="P17" t="n">
-        <v>527</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>htan2-dcc.htan2_isbcgcbq_current_release.ID_Provenance_Chain</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>HTAN2</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>ID_Provenance_Chain_current</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>ID_Provenance_Chain_r8</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>This table contains biospecimen and participant IDs for each HTAN2 data file. This table was created in July 2026 and uploaded July 2026 and corresponds to the HTAN Phase 2 Data Release 8.0.</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>HTAN PHASE 2 ID PROVENANCE CHAIN</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>current</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>htan2</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>metadata</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>NULL</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>htan</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>file_metadata</t>
-        </is>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>r8</t>
-        </is>
-      </c>
-      <c r="O18" t="n">
-        <v>65</v>
-      </c>
-      <c r="P18" t="n">
         <v>65</v>
       </c>
     </row>

</xml_diff>